<commit_message>
Skill para qualquer segmento da CAT 68: demo multissegmento, README com anexos cobertos e limites
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/modelo-RPA/resultado_levantamento.xlsx
+++ b/exemplos/modelo-RPA/resultado_levantamento.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anexo II (notas selecionadas)'!$A$1:$AI$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumo por produto'!$A$1:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anexo II (notas selecionadas)'!$A$1:$AI$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumo por produto'!$A$1:$N$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pendências'!$A$1:$H$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cliente: DROGARIA EXEMPLO LTDA</t>
+          <t>Cliente: COMERCIAL EXEMPLO LTDA</t>
         </is>
       </c>
     </row>
@@ -505,35 +505,35 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Itens triados: 5 (R$ 683,00 em estoque) | linhas de alocação: 6</t>
+          <t>Itens triados: 6 (R$ 4.251,00 em estoque) | linhas de alocação: 8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Situação da localização: Confirmado: 5</t>
+          <t>Situação da localização: Confirmado: 6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CRÉDITO TOTAL (Anexo IV): R$ 175,77 em 5 mercadorias. É o valor do lançamento: soma de todo o crédito calculado pela fórmula do anexo, com as premissas e observações registradas.</t>
+          <t>CRÉDITO TOTAL (Anexo IV): R$ 1.078,19 em 6 mercadorias. É o valor do lançamento: soma de todo o crédito calculado pela fórmula do anexo, com as premissas e observações registradas.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Composição: soma das linhas R$ 175,77 + ajuste do piso zero por mercadoria R$ 0,00 = R$ 175,77. Com VlMerc = vProd (sem descontar o desconto da nota) o crédito seria R$ 175,77.</t>
+          <t>Composição: soma das linhas R$ 1.078,19 + ajuste do piso zero por mercadoria R$ 0,00 = R$ 1.078,19. Com VlMerc = vProd (sem descontar o desconto da nota) o crédito seria R$ 1.078,19.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Observações do cálculo: R$ 104,33 do total em 3 mercadorias têm premissa a documentar: combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico (3). Detalhe nas abas Anexo II (observações do cálculo) e Pendências.</t>
+          <t>Observações do cálculo: R$ 250,75 do total em 3 mercadorias têm premissa a documentar: combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico (3). Detalhe nas abas Anexo II (observações do cálculo) e Pendências.</t>
         </is>
       </c>
     </row>
@@ -582,14 +582,14 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Entrada: só a data de emissão; sem registro de entrada: 6 (linhas de nota).</t>
+          <t>Entrada: só a data de emissão; sem registro de entrada: 8 (linhas de nota).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PONTOS EM ABERTO (não validados juridicamente; mostrados com o efeito): piso zero por mercadoria (ajuste R$ 0,00 no total); VlMerc líquido de desconto (com vProd o crédito seria R$ 175,77); FCP com base própria calculado em cada base; analogias do Anexo IV; a parcela do art. 3º, §4º (CAT 75/08) não é identificada nem deduzida.</t>
+          <t>PONTOS EM ABERTO (não validados juridicamente; mostrados com o efeito): piso zero por mercadoria (ajuste R$ 0,00 no total); VlMerc líquido de desconto (com vProd o crédito seria R$ 1.078,19); FCP com base própria calculado em cada base; analogias do Anexo IV; a parcela do art. 3º, §4º (CAT 75/08) não é identificada nem deduzida.</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI7"/>
+  <dimension ref="A1:AI9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1145,21 +1145,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOSARTANA</t>
+          <t>LAMPADA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30049069</t>
+          <t>85395200</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1300100</t>
+          <t>0900100</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1194,13 +1194,13 @@
         <v>10</v>
       </c>
       <c r="M3" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="N3" t="n">
-        <v>114.8</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>20.66</v>
+        <v>18.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>LOSARTANA POTASSICA 50MG C/30 COMP</t>
+          <t>LAMPADA LED BULBO 9W BIVOLT</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
@@ -1248,28 +1248,28 @@
       <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>descrição com dose/forma farmacêutica e NCM de medicamento; CEST da nota 13.001.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
+          <t>termo da descrição legal na descrição do produto: LAMPA; CEST da nota 09.001.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOSARTANA</t>
+          <t>LAMPADA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30049069</t>
+          <t>85395200</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1300100</t>
+          <t>0900100</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1301,16 +1301,16 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="M4" t="n">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="N4" t="n">
-        <v>168</v>
+        <v>490</v>
       </c>
       <c r="P4" t="n">
-        <v>30.24</v>
+        <v>88.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>LOSARTANA POTASSICA 50MG C/30 COMP</t>
+          <t>LAMPADA LED BULBO 9W BIVOLT</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1366,28 +1366,28 @@
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>descrição com dose/forma farmacêutica e NCM de medicamento; CEST da nota 13.001.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
+          <t>termo da descrição legal na descrição do produto: LAMPA; CEST da nota 09.001.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PARACETAMOL</t>
+          <t>SUCO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30049069</t>
+          <t>20096100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1300100</t>
+          <t>1701000</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1419,16 +1419,16 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="M5" t="n">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="N5" t="n">
-        <v>252</v>
+        <v>319.2</v>
       </c>
       <c r="P5" t="n">
-        <v>45.36</v>
+        <v>57.46</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>PARACETAMOL 750MG C/20 COMP</t>
+          <t>SUCO DE UVA INTEGRAL 1L</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
@@ -1476,24 +1476,28 @@
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>descrição com dose/forma farmacêutica e NCM de medicamento; CEST da nota 13.001.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
+          <t>termo da descrição legal na descrição do produto: SUCO; CEST da nota 17.010.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAMADEIRA</t>
+          <t>SUCO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>39241000</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>20096100</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1701000</t>
+        </is>
+      </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1514,7 +1518,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1525,16 +1529,16 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="M6" t="n">
-        <v>84</v>
+        <v>216</v>
       </c>
       <c r="N6" t="n">
-        <v>117.6</v>
+        <v>302.4</v>
       </c>
       <c r="P6" t="n">
-        <v>21.17</v>
+        <v>54.43</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1553,21 +1557,21 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>7890000000046</t>
+          <t>7890000000039</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>MAMADEIRA BICO DE SILICONE 240ML</t>
+          <t>SUCO DE UVA INTEGRAL 1L</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>01/01/2026</t>
         </is>
       </c>
       <c r="W6" t="n">
-        <v>84</v>
+        <v>216</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1590,7 +1594,7 @@
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>termo da descrição legal na descrição do produto: MAMAD; exclusão: Portaria SRE-94/25 com efeito em 01/04/2026</t>
+          <t>termo da descrição legal na descrição do produto: SUCO; CEST da nota 17.010.00 igual ao do item; exclusão: Portaria SRE-64/25 com efeito em 01/01/2026</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1667,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>7890000000053</t>
+          <t>7890000000046</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1700,8 +1704,228 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TINTA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>32091010</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2400100</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>18</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>35260822222222000122550010000010051079585953</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1260</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1764</v>
+      </c>
+      <c r="P8" t="n">
+        <v>317.52</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>C = BC ST x Alíquota interna</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>7890000000053</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>1260</v>
+      </c>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>ST da nota (pICMSST + pFCPST)</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>só a data de emissão; sem registro de entrada</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>termo da descrição legal na descrição do produto: TINTA; CEST da nota 24.001.00 igual ao do item; exclusão: Portaria SRE-34/26 com efeito em 01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PNEU</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>40111000</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1600100</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>18</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>35260822222222000122550010000010051079585953</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>10</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1920</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2688</v>
+      </c>
+      <c r="P9" t="n">
+        <v>483.84</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>C = BC ST x Alíquota interna</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>7890000000060</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>PNEU NOVO ARO 15 195/60R15</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="W9" t="n">
+        <v>1920</v>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>ST da nota (pICMSST + pFCPST)</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>só a data de emissão; sem registro de entrada</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>termo da descrição legal na descrição do produto: NOVO, PNEU; CEST da nota 16.001.00 igual ao do item; exclusão: Portaria SRE-34/26 com efeito em 01/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AI7"/>
+  <autoFilter ref="A1:AI9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1712,7 +1936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1862,7 +2086,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOSARTANA</t>
+          <t>LAMPADA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1872,7 +2096,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LOSARTANA POTASSICA 50MG C/30 COMP</t>
+          <t>LAMPADA LED BULBO 9W BIVOLT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1881,25 +2105,25 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>202</v>
+        <v>423</v>
       </c>
       <c r="G3" t="n">
-        <v>282.8</v>
+        <v>592.2</v>
       </c>
       <c r="H3" t="n">
-        <v>50.9</v>
+        <v>106.6</v>
       </c>
       <c r="I3" t="n">
-        <v>8.08</v>
+        <v>7.05</v>
       </c>
       <c r="J3" t="n">
-        <v>11.312</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>2.036</v>
+        <v>1.7767</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -1918,7 +2142,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PARACETAMOL</t>
+          <t>SUCO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1928,7 +2152,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PARACETAMOL 750MG C/20 COMP</t>
+          <t>SUCO DE UVA INTEGRAL 1L</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1937,40 +2161,44 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F4" t="n">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="G4" t="n">
-        <v>252</v>
+        <v>621.6</v>
       </c>
       <c r="H4" t="n">
-        <v>45.36</v>
+        <v>111.89</v>
       </c>
       <c r="I4" t="n">
-        <v>6</v>
+        <v>9.25</v>
       </c>
       <c r="J4" t="n">
-        <v>8.4</v>
+        <v>12.95</v>
       </c>
       <c r="K4" t="n">
-        <v>1.512</v>
+        <v>2.331</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Crédito</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
+          <t>Crédito com observações</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MAMADEIRA</t>
+          <t>SHAMPOO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1980,7 +2208,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MAMADEIRA BICO DE SILICONE 240ML</t>
+          <t>SHAMPOO ANTICASPA 400ML</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1989,44 +2217,40 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
-        <v>84</v>
+        <v>103.5</v>
       </c>
       <c r="G5" t="n">
-        <v>117.6</v>
+        <v>144.9</v>
       </c>
       <c r="H5" t="n">
-        <v>21.17</v>
+        <v>26.08</v>
       </c>
       <c r="I5" t="n">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="J5" t="n">
-        <v>19.6</v>
+        <v>16.1</v>
       </c>
       <c r="K5" t="n">
-        <v>3.5283</v>
+        <v>2.8978</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Crédito com observações</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
-        </is>
-      </c>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHAMPOO</t>
+          <t>TINTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2036,34 +2260,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SHAMPOO ANTICASPA 400ML</t>
+          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>103.5</v>
+        <v>1260</v>
       </c>
       <c r="G6" t="n">
-        <v>144.9</v>
+        <v>1764</v>
       </c>
       <c r="H6" t="n">
-        <v>26.08</v>
+        <v>317.52</v>
       </c>
       <c r="I6" t="n">
-        <v>11.5</v>
+        <v>180</v>
       </c>
       <c r="J6" t="n">
-        <v>16.1</v>
+        <v>252</v>
       </c>
       <c r="K6" t="n">
-        <v>2.8978</v>
+        <v>45.36</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -2075,8 +2299,60 @@
       </c>
       <c r="N6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PNEU</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7890000000060</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PNEU NOVO ARO 15 195/60R15</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1920</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2688</v>
+      </c>
+      <c r="H7" t="n">
+        <v>483.84</v>
+      </c>
+      <c r="I7" t="n">
+        <v>320</v>
+      </c>
+      <c r="J7" t="n">
+        <v>448</v>
+      </c>
+      <c r="K7" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:N7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2087,7 +2363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2142,7 +2418,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2172,7 +2448,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2198,7 +2474,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2224,7 +2500,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2250,7 +2526,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -2276,7 +2552,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2302,7 +2578,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -2328,7 +2604,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -2354,7 +2630,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -2380,7 +2656,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2406,7 +2682,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.71</v>
+        <v>20.89</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2432,7 +2708,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.71</v>
+        <v>20.96</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2458,7 +2734,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2472,7 +2748,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2 mercadorias com crédito</t>
+          <t>1 mercadorias com crédito</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2764,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2514,7 +2790,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2540,7 +2816,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2566,7 +2842,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2592,7 +2868,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2618,7 +2894,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2644,7 +2920,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2670,7 +2946,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2696,7 +2972,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2722,7 +2998,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3.93</v>
+        <v>2.17</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2748,7 +3024,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4.02</v>
+        <v>2.21</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2761,6 +3037,322 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1/12</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2 mercadorias com crédito</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2/12</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>3/12</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>01/2027</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>4/12</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>02/2027</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>5/12</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>6/12</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>8/12</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>11/12</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>09/2027</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2876,7 +3468,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>104.33</v>
+        <v>250.75</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Triagem pela descricao com itens que continuam na ST; panorama da CAT 68; guia 'o que enviar'; demo com sorvete e eletrodomestico
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/modelo-RPA/resultado_levantamento.xlsx
+++ b/exemplos/modelo-RPA/resultado_levantamento.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendências" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anexo II (notas selecionadas)'!$A$1:$AI$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumo por produto'!$A$1:$N$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anexo II (notas selecionadas)'!$A$1:$AI$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Resumo por produto'!$A$1:$N$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pendências'!$A$1:$H$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,35 +505,35 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Itens triados: 6 (R$ 4.251,00 em estoque) | linhas de alocação: 8</t>
+          <t>Itens triados: 8 (R$ 4.446,00 em estoque) | linhas de alocação: 11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Situação da localização: Confirmado: 6</t>
+          <t>Situação da localização: Confirmado: 8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CRÉDITO TOTAL (Anexo IV): R$ 1.078,19 em 6 mercadorias. É o valor do lançamento: soma de todo o crédito calculado pela fórmula do anexo, com as premissas e observações registradas.</t>
+          <t>CRÉDITO TOTAL (Anexo IV): R$ 1.127,46 em 8 mercadorias. É o valor do lançamento: soma de todo o crédito calculado pela fórmula do anexo, com as premissas e observações registradas.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Composição: soma das linhas R$ 1.078,19 + ajuste do piso zero por mercadoria R$ 0,00 = R$ 1.078,19. Com VlMerc = vProd (sem descontar o desconto da nota) o crédito seria R$ 1.078,19.</t>
+          <t>Composição: soma das linhas R$ 1.127,46 + ajuste do piso zero por mercadoria R$ 0,00 = R$ 1.127,46. Com VlMerc = vProd (sem descontar o desconto da nota) o crédito seria R$ 1.127,46.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Observações do cálculo: R$ 250,75 do total em 3 mercadorias têm premissa a documentar: combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico (3). Detalhe nas abas Anexo II (observações do cálculo) e Pendências.</t>
+          <t>Observações do cálculo: R$ 368,94 do total em 5 mercadorias têm premissa a documentar: combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico (5). Detalhe nas abas Anexo II (observações do cálculo) e Pendências.</t>
         </is>
       </c>
     </row>
@@ -582,14 +582,14 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Entrada: só a data de emissão; sem registro de entrada: 8 (linhas de nota).</t>
+          <t>Entrada: só a data de emissão; sem registro de entrada: 11 (linhas de nota).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PONTOS EM ABERTO (não validados juridicamente; mostrados com o efeito): piso zero por mercadoria (ajuste R$ 0,00 no total); VlMerc líquido de desconto (com vProd o crédito seria R$ 1.078,19); FCP com base própria calculado em cada base; analogias do Anexo IV; a parcela do art. 3º, §4º (CAT 75/08) não é identificada nem deduzida.</t>
+          <t>PONTOS EM ABERTO (não validados juridicamente; mostrados com o efeito): piso zero por mercadoria (ajuste R$ 0,00 no total); VlMerc líquido de desconto (com vProd o crédito seria R$ 1.127,46); FCP com base própria calculado em cada base; analogias do Anexo IV; a parcela do art. 3º, §4º (CAT 75/08) não é identificada nem deduzida.</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AI12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1643,16 +1643,16 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>103.5</v>
+        <v>115</v>
       </c>
       <c r="N7" t="n">
-        <v>144.9</v>
+        <v>161</v>
       </c>
       <c r="P7" t="n">
-        <v>26.08</v>
+        <v>28.98</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="W7" t="n">
-        <v>103.5</v>
+        <v>115</v>
       </c>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
@@ -1707,21 +1707,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TINTA</t>
+          <t>SHAMPOO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32091010</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2400100</t>
-        </is>
-      </c>
+          <t>33051000</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1733,16 +1729,16 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>35260822222222000122550010000010051079585953</t>
+          <t>35251211111111000111550010000010021079348380</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1753,16 +1749,16 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M8" t="n">
-        <v>1260</v>
+        <v>66</v>
       </c>
       <c r="N8" t="n">
-        <v>1764</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>317.52</v>
+        <v>16.63</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1771,35 +1767,43 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>Anexo IV: RPA/RPA, retenção por substituto anterior ao fornecedor (analogia: art. 4º e linha SN/substituto anterior), sem redução</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Observação do cálculo (já somada ao total): combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7890000000053</t>
+          <t>7890000000046</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
+          <t>SHAMPOO ANTICASPA 400ML</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="W8" t="n">
-        <v>1260</v>
-      </c>
-      <c r="Z8" t="inlineStr"/>
+        <v>66</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>ST da nota (pICMSST + pFCPST)</t>
+          <t>ST retido anteriormente (pST, já inclui FCP)</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
@@ -1810,28 +1814,28 @@
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>termo da descrição legal na descrição do produto: TINTA; CEST da nota 24.001.00 igual ao do item; exclusão: Portaria SRE-34/26 com efeito em 01/10/2026</t>
+          <t>termo da descrição legal na descrição do produto: XAMPU; exclusão: Portaria SRE-94/25 com efeito em 01/04/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PNEU</t>
+          <t>SORVETE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>40111000</t>
+          <t>21050010</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1600100</t>
+          <t>2300100</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1843,16 +1847,16 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>35260822222222000122550010000010051079585953</t>
+          <t>35260611111111000111550010000010061079665140</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1863,16 +1867,16 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="M9" t="n">
-        <v>1920</v>
+        <v>288</v>
       </c>
       <c r="N9" t="n">
-        <v>2688</v>
+        <v>403.2</v>
       </c>
       <c r="P9" t="n">
-        <v>483.84</v>
+        <v>72.58</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1881,35 +1885,43 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>Anexo IV: RPA/RPA, retenção por substituto anterior ao fornecedor (analogia: art. 4º e linha SN/substituto anterior), sem redução</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Observação do cálculo (já somada ao total): combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>7890000000060</t>
+          <t>7890000000077</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>PNEU NOVO ARO 15 195/60R15</t>
+          <t>SORVETE CREMOSO CHOCOLATE 2L</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="W9" t="n">
-        <v>1920</v>
-      </c>
-      <c r="Z9" t="inlineStr"/>
+        <v>288</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
       <c r="AA9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>ST da nota (pICMSST + pFCPST)</t>
+          <t>ST retido anteriormente (pST, já inclui FCP)</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
@@ -1920,12 +1932,342 @@
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr">
         <is>
+          <t>termo da descrição legal na descrição do produto: SORVE; CEST da nota 23.001.00 igual ao do item; exclusão: Portaria SRE-09/26 com efeito em 01/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FERRO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>85164000</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2104400</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>35260722222222000122550010000010071079744335</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>10</v>
+      </c>
+      <c r="M10" t="n">
+        <v>650</v>
+      </c>
+      <c r="N10" t="n">
+        <v>910</v>
+      </c>
+      <c r="P10" t="n">
+        <v>163.8</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>C = BC ST x Alíquota interna</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>7890000000084</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>FERRO ELETRICO A VAPOR 1200W</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="W10" t="n">
+        <v>650</v>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>ST da nota (pICMSST + pFCPST)</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>só a data de emissão; sem registro de entrada</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>termo da descrição legal na descrição do produto: ELETR, FERRO; CEST da nota 21.044.00 igual ao do item; exclusão: Portaria SRE-19/26 com efeito em 01/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TINTA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>32091010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2400100</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>18</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>35260822222222000122550010000010051079585953</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>12</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1080</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1512</v>
+      </c>
+      <c r="P11" t="n">
+        <v>272.16</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>C = BC ST x Alíquota interna</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>7890000000053</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="W11" t="n">
+        <v>1080</v>
+      </c>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>ST da nota (pICMSST + pFCPST)</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>só a data de emissão; sem registro de entrada</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>termo da descrição legal na descrição do produto: TINTA; CEST da nota 24.001.00 igual ao do item; exclusão: Portaria SRE-34/26 com efeito em 01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PNEU</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>40111000</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1600100</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>18</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>35260822222222000122550010000010051079585953</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>10</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>4</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1280</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1792</v>
+      </c>
+      <c r="P12" t="n">
+        <v>322.56</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>C = BC ST x Alíquota interna</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Anexo IV: RPA/RPA, retenção forn. ou antecip. adq., sem redução</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>7890000000060</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>PNEU NOVO ARO 15 195/60R15</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="W12" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>ST da nota (pICMSST + pFCPST)</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>só a data de emissão; sem registro de entrada</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr">
+        <is>
           <t>termo da descrição legal na descrição do produto: NOVO, PNEU; CEST da nota 16.001.00 igual ao do item; exclusão: Portaria SRE-34/26 com efeito em 01/10/2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI9"/>
+  <autoFilter ref="A1:AI12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1936,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2217,129 +2559,137 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
-        <v>103.5</v>
+        <v>181</v>
       </c>
       <c r="G5" t="n">
-        <v>144.9</v>
+        <v>253.4</v>
       </c>
       <c r="H5" t="n">
-        <v>26.08</v>
+        <v>45.61</v>
       </c>
       <c r="I5" t="n">
-        <v>11.5</v>
+        <v>11.3125</v>
       </c>
       <c r="J5" t="n">
-        <v>16.1</v>
+        <v>15.8375</v>
       </c>
       <c r="K5" t="n">
-        <v>2.8978</v>
+        <v>2.8506</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Crédito</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+          <t>Crédito com observações</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TINTA</t>
+          <t>SORVETE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7890000000053</t>
+          <t>7890000000077</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
+          <t>SORVETE CREMOSO CHOCOLATE 2L</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>1260</v>
+        <v>288</v>
       </c>
       <c r="G6" t="n">
-        <v>1764</v>
+        <v>403.2</v>
       </c>
       <c r="H6" t="n">
-        <v>317.52</v>
+        <v>72.58</v>
       </c>
       <c r="I6" t="n">
-        <v>180</v>
+        <v>18</v>
       </c>
       <c r="J6" t="n">
-        <v>252</v>
+        <v>25.2</v>
       </c>
       <c r="K6" t="n">
-        <v>45.36</v>
+        <v>4.5362</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Crédito</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
+          <t>Crédito com observações</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PNEU</t>
+          <t>FERRO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7890000000060</t>
+          <t>7890000000084</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PNEU NOVO ARO 15 195/60R15</t>
+          <t>FERRO ELETRICO A VAPOR 1200W</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/08/2026</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>1920</v>
+        <v>650</v>
       </c>
       <c r="G7" t="n">
-        <v>2688</v>
+        <v>910</v>
       </c>
       <c r="H7" t="n">
-        <v>483.84</v>
+        <v>163.8</v>
       </c>
       <c r="I7" t="n">
-        <v>320</v>
+        <v>65</v>
       </c>
       <c r="J7" t="n">
-        <v>448</v>
+        <v>91</v>
       </c>
       <c r="K7" t="n">
-        <v>80.64</v>
+        <v>16.38</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -2351,8 +2701,112 @@
       </c>
       <c r="N7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TINTA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7890000000053</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TINTA ACRILICA FOSCA BRANCA 18L</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1512</v>
+      </c>
+      <c r="H8" t="n">
+        <v>272.16</v>
+      </c>
+      <c r="I8" t="n">
+        <v>180</v>
+      </c>
+      <c r="J8" t="n">
+        <v>252</v>
+      </c>
+      <c r="K8" t="n">
+        <v>45.36</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PNEU</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7890000000060</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PNEU NOVO ARO 15 195/60R15</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1792</v>
+      </c>
+      <c r="H9" t="n">
+        <v>322.56</v>
+      </c>
+      <c r="I9" t="n">
+        <v>320</v>
+      </c>
+      <c r="J9" t="n">
+        <v>448</v>
+      </c>
+      <c r="K9" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N7"/>
+  <autoFilter ref="A1:N9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2363,7 +2817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2734,7 +3188,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2764,7 +3218,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2790,7 +3244,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2816,7 +3270,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2842,7 +3296,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2868,7 +3322,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2894,7 +3348,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2920,7 +3374,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2946,7 +3400,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2972,7 +3426,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2998,7 +3452,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2.17</v>
+        <v>3.8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -3024,7 +3478,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2.21</v>
+        <v>3.81</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -3041,7 +3495,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3050,7 +3504,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -3064,14 +3518,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2 mercadorias com crédito</t>
+          <t>1 mercadorias com crédito</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3080,7 +3534,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -3097,7 +3551,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3106,7 +3560,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -3123,7 +3577,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01/2027</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3132,7 +3586,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -3149,7 +3603,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>02/2027</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3158,7 +3612,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -3175,7 +3629,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>03/2027</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3184,7 +3638,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -3201,7 +3655,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>04/2027</t>
+          <t>01/2027</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3210,7 +3664,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -3227,7 +3681,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05/2027</t>
+          <t>02/2027</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3236,7 +3690,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -3253,7 +3707,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>03/2027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3262,7 +3716,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -3279,7 +3733,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>04/2027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3288,7 +3742,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -3305,7 +3759,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>05/2027</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3314,7 +3768,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>66.78</v>
+        <v>6.04</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3331,28 +3785,660 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1/12</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1 mercadorias com crédito</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2/12</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>3/12</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>4/12</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>5/12</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>01/2027</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>6/12</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>02/2027</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>8/12</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/12</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1/12</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2 mercadorias com crédito</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2/12</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>3/12</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>01/2027</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>4/12</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>02/2027</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>5/12</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>6/12</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>8/12</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>11/12</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>09/2027</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>12/12</t>
         </is>
       </c>
-      <c r="C37" t="n">
-        <v>66.78</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>RPA</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="C61" t="n">
+        <v>49.56</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>RPA</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>EFD Bloco E, código SP020750, "Outros Créditos", com menção à Portaria CAT 28/2020</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3464,11 +4550,11 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3 mercadoria(s): combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
+          <t>5 mercadoria(s): combinação não listada no Anexo IV: valor por analogia, sem fundamento oficial específico</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>250.75</v>
+        <v>368.94</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>

</xml_diff>